<commit_message>
Fixed minor problems in PCBs files
</commit_message>
<xml_diff>
--- a/Electronics/PCBs/Main/BOM.xlsx
+++ b/Electronics/PCBs/Main/BOM.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_Board1_PCB-V1_2026-03-05" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_Board1_PCB-V1_2026-03-30" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -211,7 +211,7 @@
     <t>1uF</t>
   </si>
   <si>
-    <t>CINR1,CVREF</t>
+    <t>CINR1,CUPEN,CVREF</t>
   </si>
   <si>
     <t>CL10A105KO8NNNC</t>
@@ -1261,7 +1261,7 @@
         <v>64</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" t="s">
         <v>65</v>

</xml_diff>

<commit_message>
Main PCB - V1.1
- Switched GPIO48 and GPIO46
- Added CUPEN capacitor
- Fixed audio low-pass filter and gain
- Reduced Wi-Fi antenna EMI in audio
</commit_message>
<xml_diff>
--- a/Electronics/PCBs/Main/BOM.xlsx
+++ b/Electronics/PCBs/Main/BOM.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_Board1_PCB-V1_2026-03-30" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_Board1_PCB-V1_2026-04-29" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="187">
   <si>
     <t>No.</t>
   </si>
@@ -124,100 +124,103 @@
     <t>5</t>
   </si>
   <si>
-    <t>47nF</t>
-  </si>
-  <si>
-    <t>CASIG</t>
+    <t>10uF</t>
+  </si>
+  <si>
+    <t>CAVDD2,CCH340,CDVDD2,CESP2</t>
   </si>
   <si>
     <t>C0603</t>
   </si>
   <si>
-    <t>CL10B473KB8NNNC</t>
+    <t>CL10A106MA8NRNC</t>
   </si>
   <si>
     <t>SAMSUNG(三星)</t>
   </si>
   <si>
-    <t>C1622</t>
+    <t>C96446</t>
   </si>
   <si>
     <t>6</t>
   </si>
   <si>
-    <t>10uF</t>
-  </si>
-  <si>
-    <t>CAVDD2,CCH340,CDVDD2,CESP2</t>
-  </si>
-  <si>
-    <t>CL10A106MA8NRNC</t>
-  </si>
-  <si>
-    <t>C96446</t>
+    <t>100nF</t>
+  </si>
+  <si>
+    <t>CAVDD,CAVDD1,CCAM14,CCSI_RST,CDVDD1,CESP1,CINL,CSPKR</t>
+  </si>
+  <si>
+    <t>CC0603KRX7R9BB104</t>
+  </si>
+  <si>
+    <t>YAGEO(国巨)</t>
+  </si>
+  <si>
+    <t>C14663</t>
   </si>
   <si>
     <t>7</t>
   </si>
   <si>
-    <t>100nF</t>
-  </si>
-  <si>
-    <t>CAVDD,CAVDD1,CCAM14,CCSI_RST,CDVDD1,CESP1,CINL,CINR2,CSPKR</t>
-  </si>
-  <si>
-    <t>CC0603KRX7R9BB104</t>
-  </si>
-  <si>
-    <t>YAGEO(国巨)</t>
-  </si>
-  <si>
-    <t>C14663</t>
+    <t>15pF</t>
+  </si>
+  <si>
+    <t>CCAM8</t>
+  </si>
+  <si>
+    <t>CL10C150JB8NNNC</t>
+  </si>
+  <si>
+    <t>C1644</t>
   </si>
   <si>
     <t>8</t>
   </si>
   <si>
-    <t>15pF</t>
-  </si>
-  <si>
-    <t>CCAM8</t>
-  </si>
-  <si>
-    <t>CL10C150JB8NNNC</t>
-  </si>
-  <si>
-    <t>C1644</t>
+    <t>CH340C</t>
+  </si>
+  <si>
+    <t>SOP-16_L10.0-W3.9-P1.27-LS6.0-BL</t>
+  </si>
+  <si>
+    <t>WCH(南京沁恒)</t>
+  </si>
+  <si>
+    <t>C84681</t>
   </si>
   <si>
     <t>9</t>
   </si>
   <si>
-    <t>CH340C</t>
-  </si>
-  <si>
-    <t>SOP-16_L10.0-W3.9-P1.27-LS6.0-BL</t>
-  </si>
-  <si>
-    <t>WCH(南京沁恒)</t>
-  </si>
-  <si>
-    <t>C84681</t>
+    <t>1uF</t>
+  </si>
+  <si>
+    <t>CINR1,CUPEN1,CVREF</t>
+  </si>
+  <si>
+    <t>CL10A105KO8NNNC</t>
+  </si>
+  <si>
+    <t>C1592</t>
   </si>
   <si>
     <t>10</t>
   </si>
   <si>
-    <t>1uF</t>
-  </si>
-  <si>
-    <t>CINR1,CUPEN,CVREF</t>
-  </si>
-  <si>
-    <t>CL10A105KO8NNNC</t>
-  </si>
-  <si>
-    <t>C1592</t>
+    <t>10nF</t>
+  </si>
+  <si>
+    <t>CINR2</t>
+  </si>
+  <si>
+    <t>0603B103K500NT</t>
+  </si>
+  <si>
+    <t>FH(风华)</t>
+  </si>
+  <si>
+    <t>C57112</t>
   </si>
   <si>
     <t>11</t>
@@ -430,7 +433,7 @@
     <t>10kΩ</t>
   </si>
   <si>
-    <t>RDTR,RRTS,RUPEN</t>
+    <t>RDTR,RRTS,RUPEN1</t>
   </si>
   <si>
     <t>0603WAF1002T5E</t>
@@ -445,6 +448,21 @@
     <t>24</t>
   </si>
   <si>
+    <t>22kΩ</t>
+  </si>
+  <si>
+    <t>RPAM</t>
+  </si>
+  <si>
+    <t>0603WAF2202T5E</t>
+  </si>
+  <si>
+    <t>C31850</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
     <t>4.7kΩ</t>
   </si>
   <si>
@@ -457,7 +475,7 @@
     <t>C23162</t>
   </si>
   <si>
-    <t>25</t>
+    <t>26</t>
   </si>
   <si>
     <t>2.2kΩ</t>
@@ -472,7 +490,7 @@
     <t>C4190</t>
   </si>
   <si>
-    <t>26</t>
+    <t>27</t>
   </si>
   <si>
     <t>1.25mm-2P ZZ-MS</t>
@@ -490,7 +508,7 @@
     <t>C5368706</t>
   </si>
   <si>
-    <t>27</t>
+    <t>28</t>
   </si>
   <si>
     <t>TYPE-C16PIN</t>
@@ -505,7 +523,7 @@
     <t>C393939</t>
   </si>
   <si>
-    <t>28</t>
+    <t>29</t>
   </si>
   <si>
     <t>USBLC6-2SC6</t>
@@ -523,7 +541,7 @@
     <t>C7519</t>
   </si>
   <si>
-    <t>29</t>
+    <t>30</t>
   </si>
   <si>
     <t>XC6206-1.2V</t>
@@ -541,7 +559,7 @@
     <t>C49446790</t>
   </si>
   <si>
-    <t>30</t>
+    <t>31</t>
   </si>
   <si>
     <t>XC6206-2.8V</t>
@@ -930,7 +948,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -1101,7 +1119,7 @@
         <v>36</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
@@ -1133,7 +1151,7 @@
         <v>43</v>
       </c>
       <c r="B7">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
         <v>44</v>
@@ -1151,10 +1169,10 @@
         <v>46</v>
       </c>
       <c r="H7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="I7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J7" t="s">
         <v>17</v>
@@ -1162,28 +1180,28 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B8">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
         <v>39</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H8" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="I8" t="s">
         <v>53</v>
@@ -1203,19 +1221,19 @@
         <v>55</v>
       </c>
       <c r="D9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" t="s">
         <v>56</v>
       </c>
-      <c r="E9" t="s">
-        <v>39</v>
-      </c>
       <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
         <v>55</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>57</v>
-      </c>
-      <c r="H9" t="s">
-        <v>41</v>
       </c>
       <c r="I9" t="s">
         <v>58</v>
@@ -1229,25 +1247,25 @@
         <v>59</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10" t="s">
         <v>60</v>
       </c>
       <c r="D10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" t="s">
         <v>60</v>
       </c>
-      <c r="E10" t="s">
-        <v>61</v>
-      </c>
-      <c r="F10" t="s">
-        <v>14</v>
-      </c>
       <c r="G10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H10" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="I10" t="s">
         <v>63</v>
@@ -1261,7 +1279,7 @@
         <v>64</v>
       </c>
       <c r="B11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C11" t="s">
         <v>65</v>
@@ -1279,10 +1297,10 @@
         <v>67</v>
       </c>
       <c r="H11" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="I11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J11" t="s">
         <v>17</v>
@@ -1290,31 +1308,31 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B12">
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F12" t="s">
         <v>14</v>
       </c>
       <c r="G12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H12" t="s">
         <v>28</v>
       </c>
       <c r="I12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J12" t="s">
         <v>17</v>
@@ -1322,31 +1340,31 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B13">
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
       </c>
       <c r="G13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H13" t="s">
         <v>28</v>
       </c>
       <c r="I13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J13" t="s">
         <v>17</v>
@@ -1354,31 +1372,31 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B14">
         <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F14" t="s">
         <v>14</v>
       </c>
       <c r="G14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H14" t="s">
         <v>28</v>
       </c>
       <c r="I14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J14" t="s">
         <v>17</v>
@@ -1386,31 +1404,31 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F15" t="s">
         <v>14</v>
       </c>
       <c r="G15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H15" t="s">
         <v>28</v>
       </c>
       <c r="I15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J15" t="s">
         <v>17</v>
@@ -1418,31 +1436,31 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E16" t="s">
+        <v>93</v>
+      </c>
+      <c r="F16" t="s">
         <v>91</v>
       </c>
-      <c r="E16" t="s">
-        <v>92</v>
-      </c>
-      <c r="F16" t="s">
-        <v>90</v>
-      </c>
       <c r="G16" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J16" t="s">
         <v>17</v>
@@ -1450,31 +1468,31 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B17">
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D17" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E17" t="s">
         <v>39</v>
       </c>
       <c r="F17" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H17" t="s">
         <v>41</v>
       </c>
       <c r="I17" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J17" t="s">
         <v>17</v>
@@ -1482,31 +1500,31 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B18">
         <v>2</v>
       </c>
       <c r="C18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F18" t="s">
         <v>14</v>
       </c>
       <c r="G18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J18" t="s">
         <v>17</v>
@@ -1514,31 +1532,31 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D19" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F19" t="s">
         <v>14</v>
       </c>
       <c r="G19" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J19" t="s">
         <v>17</v>
@@ -1546,31 +1564,31 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B20">
         <v>3</v>
       </c>
       <c r="C20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F20" t="s">
         <v>14</v>
       </c>
       <c r="G20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J20" t="s">
         <v>17</v>
@@ -1578,31 +1596,31 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D21" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F21" t="s">
         <v>14</v>
       </c>
       <c r="G21" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J21" t="s">
         <v>17</v>
@@ -1610,31 +1628,31 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B22">
         <v>2</v>
       </c>
       <c r="C22" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D22" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E22" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
       </c>
       <c r="G22" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H22" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I22" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J22" t="s">
         <v>17</v>
@@ -1642,31 +1660,31 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B23">
         <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D23" t="s">
+        <v>134</v>
+      </c>
+      <c r="E23" t="s">
+        <v>135</v>
+      </c>
+      <c r="F23" t="s">
         <v>133</v>
       </c>
-      <c r="E23" t="s">
-        <v>134</v>
-      </c>
-      <c r="F23" t="s">
-        <v>132</v>
-      </c>
       <c r="G23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H23" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="I23" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J23" t="s">
         <v>17</v>
@@ -1674,31 +1692,31 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B24">
         <v>3</v>
       </c>
       <c r="C24" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D24" t="s">
+        <v>140</v>
+      </c>
+      <c r="E24" t="s">
+        <v>135</v>
+      </c>
+      <c r="F24" t="s">
         <v>139</v>
       </c>
-      <c r="E24" t="s">
-        <v>134</v>
-      </c>
-      <c r="F24" t="s">
-        <v>138</v>
-      </c>
       <c r="G24" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H24" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I24" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J24" t="s">
         <v>17</v>
@@ -1706,31 +1724,31 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B25">
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D25" t="s">
+        <v>146</v>
+      </c>
+      <c r="E25" t="s">
+        <v>135</v>
+      </c>
+      <c r="F25" t="s">
         <v>145</v>
       </c>
-      <c r="E25" t="s">
-        <v>134</v>
-      </c>
-      <c r="F25" t="s">
-        <v>144</v>
-      </c>
       <c r="G25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H25" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I25" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J25" t="s">
         <v>17</v>
@@ -1738,31 +1756,31 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B26">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D26" t="s">
+        <v>151</v>
+      </c>
+      <c r="E26" t="s">
+        <v>135</v>
+      </c>
+      <c r="F26" t="s">
         <v>150</v>
       </c>
-      <c r="E26" t="s">
-        <v>134</v>
-      </c>
-      <c r="F26" t="s">
-        <v>149</v>
-      </c>
       <c r="G26" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H26" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I26" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J26" t="s">
         <v>17</v>
@@ -1770,28 +1788,28 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B27">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D27" t="s">
+        <v>156</v>
+      </c>
+      <c r="E27" t="s">
+        <v>135</v>
+      </c>
+      <c r="F27" t="s">
         <v>155</v>
       </c>
-      <c r="E27" t="s">
-        <v>156</v>
-      </c>
-      <c r="F27" t="s">
-        <v>14</v>
-      </c>
       <c r="G27" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="H27" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I27" t="s">
         <v>158</v>
@@ -1823,10 +1841,10 @@
         <v>160</v>
       </c>
       <c r="H28" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="I28" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J28" t="s">
         <v>17</v>
@@ -1834,28 +1852,28 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B29">
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D29" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E29" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F29" t="s">
         <v>14</v>
       </c>
       <c r="G29" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H29" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="I29" t="s">
         <v>169</v>
@@ -1919,17 +1937,49 @@
         <v>177</v>
       </c>
       <c r="H31" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="I31" t="s">
+        <v>181</v>
+      </c>
+      <c r="J31" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>182</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>183</v>
+      </c>
+      <c r="D32" t="s">
+        <v>184</v>
+      </c>
+      <c r="E32" t="s">
+        <v>185</v>
+      </c>
+      <c r="F32" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" t="s">
+        <v>183</v>
+      </c>
+      <c r="H32" t="s">
         <v>180</v>
       </c>
-      <c r="J31" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="I32" t="s">
+        <v>186</v>
+      </c>
+      <c r="J32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>